<commit_message>
Next make is Sinotruk C7H: docs/13 + checklist, pre-filled sinotruk_c7h_template.xlsx, prepared (unapplied) make_profile SQL, docs/14 plan for the 4 app follow-ups
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/new_make_template.xlsx
+++ b/docs/templates/new_make_template.xlsx
@@ -153,22 +153,22 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Short code, CAPITALS/digits/_ (profile: SONNET_X; section: BMP; supplier: SUP-ACME)</t>
+        <t>Short code, CAPITALS/digits/_ (profile: SINOTRUK_C7H; section: BMP; supplier: SUP-ACME)</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Vehicle make exactly as it should show in CTP and Zoho Manufacturer (e.g. Sonnet). Universal parts: 'All makes'</t>
+        <t>Vehicle make exactly as it should show in CTP and Zoho Manufacturer (e.g. Sinotruk). Universal parts: 'All makes'</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Vehicle model (= Zoho Brand), e.g. X3000. Blank for universal / all-makes parts</t>
+        <t>Vehicle model (= Zoho Brand), e.g. C7H. Blank for universal / all-makes parts</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Name people see, e.g. 'Sonnet X3000'</t>
+        <t>Name people see, e.g. 'Sinotruk C7H'</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -198,12 +198,12 @@
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Zoho GL account id for sales, e.g. 'Sales - Sonnet' (onboard.py accounts lists them)</t>
+        <t>Zoho GL account id for sales, e.g. 'Sales - Sinotruk' (onboard.py accounts lists them)</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Zoho GL id for cost of sales, e.g. 'Cost of Goods Sold - Sonnet'</t>
+        <t>Zoho GL id for cost of sales, e.g. 'Cost of Goods Sold - Sinotruk'</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
@@ -263,7 +263,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Unique drawing code, e.g. SONNET_X-BMP (never SEC&lt;number&gt;: those are FAW JH6's)</t>
+        <t>Unique drawing code, e.g. SINOTRUK_C7H-BMP (never SEC&lt;number&gt;: those are FAW JH6's)</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -358,12 +358,12 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Vehicle model (= Zoho Brand), e.g. X3000. Blank for universal / all-makes parts</t>
+        <t>Vehicle model (= Zoho Brand), e.g. C7H. Blank for universal / all-makes parts</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Vehicle make exactly as it should show in CTP and Zoho Manufacturer (e.g. Sonnet). Universal parts: 'All makes'</t>
+        <t>Vehicle make exactly as it should show in CTP and Zoho Manufacturer (e.g. Sinotruk). Universal parts: 'All makes'</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
@@ -403,7 +403,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Short code, CAPITALS/digits/_ (profile: SONNET_X; section: BMP; supplier: SUP-ACME)</t>
+        <t>Short code, CAPITALS/digits/_ (profile: SINOTRUK_C7H; section: BMP; supplier: SUP-ACME)</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -423,7 +423,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Short code, CAPITALS/digits/_ (profile: SONNET_X; section: BMP; supplier: SUP-ACME)</t>
+        <t>Short code, CAPITALS/digits/_ (profile: SINOTRUK_C7H; section: BMP; supplier: SUP-ACME)</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -503,12 +503,12 @@
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Vehicle make exactly as it should show in CTP and Zoho Manufacturer (e.g. Sonnet). Universal parts: 'All makes'</t>
+        <t>Vehicle make exactly as it should show in CTP and Zoho Manufacturer (e.g. Sinotruk). Universal parts: 'All makes'</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Vehicle model (= Zoho Brand), e.g. X3000. Blank for universal / all-makes parts</t>
+        <t>Vehicle model (= Zoho Brand), e.g. C7H. Blank for universal / all-makes parts</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -583,12 +583,12 @@
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Vehicle model (= Zoho Brand), e.g. X3000. Blank for universal / all-makes parts</t>
+        <t>Vehicle model (= Zoho Brand), e.g. C7H. Blank for universal / all-makes parts</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Vehicle make exactly as it should show in CTP and Zoho Manufacturer (e.g. Sonnet). Universal parts: 'All makes'</t>
+        <t>Vehicle make exactly as it should show in CTP and Zoho Manufacturer (e.g. Sinotruk). Universal parts: 'All makes'</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
@@ -713,7 +713,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Unique drawing code, e.g. SONNET_X-BMP (never SEC&lt;number&gt;: those are FAW JH6's)</t>
+        <t>Unique drawing code, e.g. SINOTRUK_C7H-BMP (never SEC&lt;number&gt;: those are FAW JH6's)</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -1118,7 +1118,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t># SONNET_X-BMP</t>
+          <t># SINOTRUK_C7H-BMP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1197,7 +1197,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t># SONNET_X-BMP</t>
+          <t># SINOTRUK_C7H-BMP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DZ95189586</t>
+          <t>WG9725000001</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1274,12 +1274,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t># DZ95189586</t>
+          <t># WG9725000001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>pictures/DZ95189586.jpg</t>
+          <t>pictures/WG9725000001.jpg</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DZ95189586</t>
+          <t>WG9725000001</t>
         </is>
       </c>
     </row>
@@ -1475,32 +1475,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t># SONNET_X</t>
+          <t># SINOTRUK_C7H</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sonnet</t>
+          <t>Sinotruk</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>X3000</t>
+          <t>C7H</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sonnet X3000</t>
+          <t>Sinotruk C7H</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SONNET</t>
+          <t>SINOTRUK</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Sonnet Genuine</t>
+          <t>Sinotruk Genuine</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1510,12 +1510,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Sonnet</t>
+          <t>Sinotruk</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>X3000</t>
+          <t>C7H</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -1606,7 +1606,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t># X3000</t>
+          <t># C7H</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -1893,7 +1893,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t># DZ95189586</t>
+          <t># WG9725000001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2004,12 +2004,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t># DZ95189586</t>
+          <t># WG9725000001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X3000</t>
+          <t>C7H</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -2075,7 +2075,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t># DZ95189586</t>
+          <t># WG9725000001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2169,7 +2169,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t># DZ95189586</t>
+          <t># WG9725000001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>